<commit_message>
Completa mejoras de la API del restaurante
</commit_message>
<xml_diff>
--- a/docs/Roles_AmericanBites.xlsx
+++ b/docs/Roles_AmericanBites.xlsx
@@ -654,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1130,19 +1130,19 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>Mesas</t>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Menú</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Listar todas las mesas</t>
+          <t>Ver el detalle de un plato del menú</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>GET /api/v1/mesas</t>
+          <t>GET /api/v1/menu/{id}</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1165,9 +1165,9 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -1179,12 +1179,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Consultar mesas disponibles</t>
+          <t>Listar todas las mesas</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>GET /api/v1/mesas/disponibles</t>
+          <t>GET /api/v1/mesas</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1221,12 +1221,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Ver detalle de una mesa</t>
+          <t>Consultar mesas disponibles</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>GET /api/v1/mesas/{id}</t>
+          <t>GET /api/v1/mesas/disponibles</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1263,12 +1263,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Crear mesa</t>
+          <t>Ver detalle de una mesa</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>POST /api/v1/mesas</t>
+          <t>GET /api/v1/mesas/{id}</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1276,19 +1276,19 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1305,12 +1305,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Cambiar estado de una mesa</t>
+          <t>Crear mesa</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/mesas/{id}/estado</t>
+          <t>POST /api/v1/mesas</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1318,9 +1318,9 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1347,74 +1347,74 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
+          <t>Cambiar estado de una mesa</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /api/v1/mesas/{id}/estado</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Mesas</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
           <t>Eliminar mesa</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>DELETE /api/v1/mesas/{id}</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>Pedidos</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Listar todos los pedidos</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>GET /api/v1/pedidos</t>
-        </is>
-      </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -1431,12 +1431,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Ver pedidos de una mesa</t>
+          <t>Listar todos los pedidos</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>GET /api/v1/pedidos/mesa/{idMesa}</t>
+          <t>GET /api/v1/pedidos</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1473,12 +1473,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Ver detalle de un pedido</t>
+          <t>Ver pedidos de una mesa</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>GET /api/v1/pedidos/{id}</t>
+          <t>GET /api/v1/pedidos/mesa/{idMesa}</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Tomar pedido (crear pedido)</t>
+          <t>Ver detalle de un pedido</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>POST /api/v1/pedidos</t>
+          <t>GET /api/v1/pedidos/{id}</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1533,14 +1533,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1557,12 +1557,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Agregar ítem a un pedido</t>
+          <t>Tomar pedido (crear pedido)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>POST /api/v1/pedidos/{id}/items</t>
+          <t>POST /api/v1/pedidos</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1599,56 +1599,56 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
+          <t>Agregar ítem a un pedido</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/v1/pedidos/{id}/items</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Pedidos</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
           <t>Cambiar estado de un pedido</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>PATCH /api/v1/pedidos/{id}/estado</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Cuentas</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Listar todas las cuentas</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>GET /api/v1/cuentas</t>
-        </is>
-      </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -1659,14 +1659,14 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -1683,12 +1683,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Ver detalle de una cuenta</t>
+          <t>Listar todas las cuentas</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>GET /api/v1/cuentas/{id}</t>
+          <t>GET /api/v1/cuentas</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1725,12 +1725,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Ver cuenta abierta de una mesa</t>
+          <t>Ver detalle de una cuenta</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>GET /api/v1/cuentas/mesa/{idMesa}</t>
+          <t>GET /api/v1/cuentas/{id}</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1767,12 +1767,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Abrir cuenta de una mesa</t>
+          <t>Ver cuenta abierta de una mesa</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>POST /api/v1/cuentas</t>
+          <t>GET /api/v1/cuentas/mesa/{idMesa}</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1790,9 +1790,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -1809,12 +1809,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Registrar pago de una cuenta</t>
+          <t>Abrir cuenta de una mesa</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/cuentas/{id}/pago</t>
+          <t>POST /api/v1/cuentas</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1822,9 +1822,9 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -1832,9 +1832,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -1851,64 +1851,64 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
+          <t>Registrar pago de una cuenta</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /api/v1/cuentas/{id}/pago</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Cuentas</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
           <t>Cerrar una cuenta</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>PATCH /api/v1/cuentas/{id}/cerrar</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>Reservas</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Listar todas las reservas</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>GET /api/v1/reservas</t>
-        </is>
-      </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -1935,12 +1935,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Ver reservas de una mesa</t>
+          <t>Listar todas las reservas</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>GET /api/v1/reservas/mesa/{idMesa}</t>
+          <t>GET /api/v1/reservas</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1977,12 +1977,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Ver detalle de una reserva</t>
+          <t>Ver reservas de una mesa</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>GET /api/v1/reservas/{id}</t>
+          <t>GET /api/v1/reservas/mesa/{idMesa}</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -2005,9 +2005,9 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -2019,12 +2019,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Crear reserva</t>
+          <t>Ver detalle de una reserva</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>POST /api/v1/reservas</t>
+          <t>GET /api/v1/reservas/{id}</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -2042,9 +2042,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -2061,12 +2061,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Cancelar reserva</t>
+          <t>Crear reserva</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/reservas/{id}/cancelar</t>
+          <t>POST /api/v1/reservas</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -2103,35 +2103,77 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
+          <t>Cancelar reserva</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>PATCH /api/v1/reservas/{id}/cancelar</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Reservas</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
           <t>Reprogramar reserva</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>PATCH /api/v1/reservas/{id}/reprogramar</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -2191,6 +2233,7 @@
 - Platos: Eliminar plato
 - Menú: Ver el menú (solo disponibles)
 - Menú: Ver menú por categoría
+- Menú: Ver el detalle de un plato del menú
 - Mesas: Listar todas las mesas
 - Mesas: Consultar mesas disponibles
 - Mesas: Ver detalle de una mesa
@@ -2233,6 +2276,7 @@
 - Platos: Ver detalle de un plato
 - Menú: Ver el menú (solo disponibles)
 - Menú: Ver menú por categoría
+- Menú: Ver el detalle de un plato del menú
 - Mesas: Listar todas las mesas
 - Mesas: Consultar mesas disponibles
 - Mesas: Ver detalle de una mesa
@@ -2282,6 +2326,7 @@
 - Platos: Ver detalle de un plato
 - Menú: Ver el menú (solo disponibles)
 - Menú: Ver menú por categoría
+- Menú: Ver el detalle de un plato del menú
 - Mesas: Listar todas las mesas
 - Mesas: Consultar mesas disponibles
 - Mesas: Ver detalle de una mesa
@@ -2331,6 +2376,7 @@
 - Platos: Ver detalle de un plato
 - Menú: Ver el menú (solo disponibles)
 - Menú: Ver menú por categoría
+- Menú: Ver el detalle de un plato del menú
 - Mesas: Listar todas las mesas
 - Mesas: Consultar mesas disponibles
 - Mesas: Ver detalle de una mesa
@@ -2376,6 +2422,7 @@
         <is>
           <t>- Menú: Ver el menú (solo disponibles)
 - Menú: Ver menú por categoría
+- Menú: Ver el detalle de un plato del menú
 - Reservas: Ver detalle de una reserva
 - Reservas: Crear reserva
 - Reservas: Cancelar reserva
@@ -2525,7 +2572,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>MESERO/ADMIN gestionan todas las reservas. El CLIENTE solo gestiona las suyas. Una mesa debe estar DISPONIBLE para reservarse.</t>
+          <t>MESERO/ADMIN gestionan todas las reservas. El CLIENTE solo gestiona las suyas. Una mesa debe estar DISPONIBLE para reservarse. Una mesa tampoco puede tener dos reservas vigentes que se solapen (bloque de 2 horas).</t>
         </is>
       </c>
     </row>

</xml_diff>